<commit_message>
Expand QBR with sourced market and competitive review
Co-authored-by: Sahil Patni <sahilpat28@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/qbr/output/Sahil_QBR_Pipeline_Summary.xlsx
+++ b/qbr/output/Sahil_QBR_Pipeline_Summary.xlsx
@@ -10,11 +10,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sahil Line Items" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market References" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Executive Summary'!$A$1:$C$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Opportunities'!$A$1:$O$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sahil Line Items'!$A$1:$T$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Market References'!$A$1:$E$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3516,4 +3518,503 @@
   <autoFilter ref="A1:T21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Accessed</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Use</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>International Federation of Robotics, World Robotics 2025 press release</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://ifr.org/ifr-press-releases/news/global-robot-demand-in-factories-doubles-over-10-years</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Robotics market</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Rockwell Automation, 2025 State of Smart Manufacturing — APAC findings</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rockwellautomation.com/en-sg/company/news/press-releases/apac-sosm-2025.html</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Industrial / APAC market</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Interact Analysis, Machine Vision return-to-growth forecast, June 2025</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://interactanalysis.com/return-to-growth-forecast-for-machine-vision-in-2025-despite-us-tariffs/</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Machine-vision market</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Robotics Solutions Stack</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/fpga-solutions/robotics-solutions-stack</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Altera robotics</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Agilex 5 FPGA and SoC FPGA overview</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/products/fpga/agilex/5</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Altera Agilex 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>AMD, Kria KR260 robotics platform and Kria Robotics Stack</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amd.com/en/products/system-on-modules/kria/k26/robotics.html</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>AMD robotics</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Video and Vision Processing Suite</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/products/ip/po-3150/video-and-vision-processing-suite</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Altera video / vision</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>R8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Altera, FPGA AI Suite</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/products/development-tools/fpga-ai-suite</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Altera AI software</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>AMD, Kria KV260 Vision AI Starter Kit</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amd.com/en/products/system-on-modules/kria/k26/kv260-vision-starter-kit.html</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>AMD vision</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>R10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>AMD, Versal AI Edge Series</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amd.com/en/products/adaptive-socs-and-fpgas/versal/ai-edge-series.html</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>AMD AI portfolio</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>R11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Industrial solutions</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/fpga-solutions/industrial</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Altera industrial</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Agilex 5 SoC HPS features including three 2.5G TSN Ethernet MACs</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>https://docs.altera.com/r/docs/762191/current/agilextm-5-fpgas-and-socs-device-overview/additional-features-for-agilextm-5-socs</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Altera TSN / HPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>R13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>AMD, Industrial Networking solutions</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amd.com/en/solutions/industrial/industrial-networking.html</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>AMD industrial networking</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Agilex 5 Functional Safety</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>https://docs.altera.com/api/khub/documents/xhgkkZ1PZaLEHFnNiUlbNA/content</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Altera functional safety</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>AMD, Functional Safety</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amd.com/en/products/adaptive-socs-and-fpgas/technologies/functional-safety.html</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>AMD functional safety</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Agilex 3 FPGA and SoC FPGA overview</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/products/fpga/agilex/3</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Altera cost-optimized portfolio</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>R17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>AMD, Spartan UltraScale+ FPGA overview</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amd.com/en/products/adaptive-socs-and-fpgas/fpga/spartan-ultrascale-plus.html</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>AMD cost-optimized portfolio</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>R18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>AMD, Vitis unified software platform</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amd.com/en/products/software/adaptive-socs-and-fpgas/vitis.html</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>AMD development tools</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E19"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add joint distributor solution execution plan
Co-authored-by: Sahil Patni <sahilpat28@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/qbr/output/Sahil_QBR_Pipeline_Summary.xlsx
+++ b/qbr/output/Sahil_QBR_Pipeline_Summary.xlsx
@@ -11,12 +11,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sahil Line Items" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market References" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joint GTM Plan" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Executive Summary'!$A$1:$C$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Opportunities'!$A$1:$O$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sahil Line Items'!$A$1:$T$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Market References'!$A$1:$E$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Market References'!$A$1:$E$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Joint GTM Plan'!$A$1:$F$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3526,14 +3528,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="58" customWidth="1" min="2" max="2"/>
     <col width="90" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="33" customWidth="1" min="5" max="5"/>
+    <col width="37" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4013,8 +4015,323 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>R19</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Video Solutions Stack</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/fpga-solutions/video-solutions-stack</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Altera video solution stack</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>R20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Sensor Interfaces including Holoscan Sensor Bridge</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/fpga-solutions/sensory-interfaces</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Altera Holoscan / sensor interfaces</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E19"/>
+  <autoFilter ref="A1:E21"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Workstream</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Commitment</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Due</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Proposed KPI</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Altera / Sahil</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Lead program, architecture, benchmarks and DFAE coordination</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Named and charter accepted</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>NAMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Arrow</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Name robotics/AI/camera-capable joint specialist</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>≥1 named specialist</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Macnica</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Name robotics/AI/camera-capable joint specialist</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>≥1 named specialist</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Readiness</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Joint tiger team</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Verify solution access, kits, skills and benchmark playbooks</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>46248</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>≥1 robotics + ≥1 camera/AI demo path</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Targeting</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Arrow + Macnica</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Create non-duplicated joint account map</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>30 accounts: 15 per distributor</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Joint tiger team</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Run segment workshops and launch evaluations</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>46326</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>12 workshops; 8 evaluations</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Conversion</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Sales + FAE + distis</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Advance evidence-backed opportunities</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>46387</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>6 qualified; 3 Develop/Design; 2 DWINs</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>PROPOSED</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reconcile QBR with 2026 and 2027 open pipeline
Co-authored-by: Sahil Patni <sahilpat28@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/qbr/output/Sahil_QBR_Pipeline_Summary.xlsx
+++ b/qbr/output/Sahil_QBR_Pipeline_Summary.xlsx
@@ -9,16 +9,22 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sahil Line Items" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market References" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joint GTM Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline Reconciliation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Pipeline 2026" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Pipeline 2027" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sahil Line Items" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market References" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joint GTM Plan" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Executive Summary'!$A$1:$C$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Opportunities'!$A$1:$O$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sahil Line Items'!$A$1:$T$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Market References'!$A$1:$E$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Joint GTM Plan'!$A$1:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Executive Summary'!$A$1:$C$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Opportunities'!$A$1:$P$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pipeline Reconciliation'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Open Pipeline 2026'!$A$1:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Open Pipeline 2027'!$A$1:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sahil Line Items'!$A$1:$T$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Market References'!$A$1:$E$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Joint GTM Plan'!$A$1:$F$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -450,10 +456,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="44" customWidth="1" min="3" max="3"/>
   </cols>
@@ -478,174 +484,219 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Distinct opportunities</t>
+          <t>Qualified open opportunities</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Consolidated by Opportunity ID</t>
+          <t>Combined uploaded 2026 + 2027 open exports</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Product line items</t>
+          <t>Qualified open peak value</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>20</v>
+        <v>8215045</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Rows where Technical Owner = Sahil Patni</t>
+          <t>Currency absent from source</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Direct-account customers</t>
+          <t>Qualified open weighted value</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>7</v>
+        <v>2507761.25</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Distinct Account Name</t>
+          <t>Peak Value × normalized Probability</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Peak pipeline</t>
+          <t>2026 open-export opportunities</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>11815045</v>
+        <v>1</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Sum of consolidated Peak Value; currency absent</t>
+          <t>User-provided planning bucket</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Weighted pipeline</t>
+          <t>2026 open-export peak value</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>2507761.25</v>
+        <v>4125000</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Peak Value × Probability</t>
+          <t>User-provided planning bucket</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-created opportunities</t>
+          <t>2027 open-export opportunities</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Created Date in 2026</t>
+          <t>User-provided planning bucket</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-created peak value</t>
+          <t>2027 open-export peak value</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>6700000</v>
+        <v>4090045</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Peak Value</t>
+          <t>User-provided planning bucket</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026 DWIN-dated opportunities</t>
+          <t>Identify outside open exports</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Scheduled DWIN date in 2026; not achieved DWIN</t>
+          <t>Master-report opportunities absent from both open exports</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026 DWIN-dated peak value</t>
+          <t>Identify peak value</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>5305000</v>
+        <v>3600000</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Peak Value</t>
+          <t>0% probability in master report</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026 annual target</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>INPUT REQUIRED</t>
-        </is>
+          <t>Total discovered opportunities</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>14</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Not present in source</t>
+          <t>Qualified open + Identify</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>Total discovered peak value</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>11815045</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Qualified open + Identify</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Product line items</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Rows where Technical Owner = Sahil Patni</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026 annual target</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>INPUT REQUIRED</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Not present in source</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>YTD actual achievement</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>INPUT REQUIRED</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Not present in source</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C12"/>
+  <autoFilter ref="A1:C15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -656,7 +707,1316 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:P15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="43" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="52" customWidth="1" min="15" max="15"/>
+    <col width="48" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Open Pipeline Bucket</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Opportunity ID</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Opportunity</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Probability (%)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Design Win Date</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Created Date</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Production Start Date</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Vertical</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Peak Value</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Weighted Value</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Product Count</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Products</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Suggested Next Gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>006Ui00001cftdL</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Outdu Mediatech Private Limited</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Intelligent Sense _Response Solution_AI</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Define</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>46316</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>45882</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>46679</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Broadcast</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>4125000</v>
+      </c>
+      <c r="M2" s="3" t="n">
+        <v>1031250</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Agilex? 5 FPGA D-Series 064 (B32B) A5DD064AB32BI2V</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Freeze architecture/BOM and evaluation plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>006Ui000029ckMz</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>JUNIPER NETWORKS</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>CFPGA_PCIe Gen1</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Develop</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>46437</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>46075</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>46611</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Networking and Data Center OEM (IHV, ISV, SI, VAR)</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>900000</v>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>450000</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Cyclone® V GX FPGA 5CGXC7 (F31) 5CGXFC7D6F31I7N</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Close validation plan and design-freeze evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>006Ui00002SuI1A</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Outdu Mediatech Private Limited</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Long Range Tracking System</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Define</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>46463</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>46028</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>47017</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Broadcast</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>825000</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>206250</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Agilex? 5 FPGA D-Series 064 (B32B) A5DD064AB32BI3V</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Freeze architecture/BOM and evaluation plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>006Ui000023SJPy</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>EMERSON INNOVATION CENTER - PUNE</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>RX3i CEP002</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Define</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>46372</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>46044</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>46491</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>775000</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>193750</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>Agilex? 3 FPGA C-Series 100 (B23C) A3CW100BB23CI6S
+Cyclone® V ST FPGA 5CSTD5 (F31) 5CSTFD5D5F31I7N</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Freeze architecture/BOM and evaluation plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>006Ui00002VpuJp</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>GE HEALTHCARE</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Anesthesia Controller_X</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Define</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>46535</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>46189</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>46764</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Medical</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>500000</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>125000</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>Agilex? 5 FPGA E-Series 028B (B23A) A5ED028BB23AI5S</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>Freeze architecture/BOM and evaluation plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>006Ui00001rc0zI</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>GE HEALTHCARE</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>CT Scanner_DCB</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Define</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>46575</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>45972</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>47296</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Medical</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="n">
+        <v>400045</v>
+      </c>
+      <c r="M7" s="3" t="n">
+        <v>100011.25</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Agilex? 3 FPGA C-Series 065 (B18A) A3CY065BB18AE6S
+Cyclone® 10 GX FPGA 10CX150 (F672) 10CX150YF672E5G</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>Freeze architecture/BOM and evaluation plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>006Ui00001YL1Wo</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Philips India Limited - Innovation Center</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>XSC/CT Scanner</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>46276</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>45770</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>46345</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Medical</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>270000</v>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>202500</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Cyclone® 10 LP FPGA 10CL120 (F780) 10CL120YF780C8G</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>Secure DW evidence and production handoff</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>006Ui00001nEdch</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>HONEYWELL TECHNOLOGY SOLUTIONS</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>micro vapour cooling system - VCS</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>46539</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>45945</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>46741</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Aerospace</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="n">
+        <v>185000</v>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>138750</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>MAX® 10 FPGA 10M04 (U324) 10M04SAU324I7G
+MAX® 10 FPGA 10M02 (U169) 10M02SCU169A7G</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>Secure DW evidence and production handoff</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>006Ui00001YKvSK</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>GE HEALTHCARE</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>SP-PDU CONTROL BOARD</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Define</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>46351</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>45732</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>46806</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Medical</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>110000</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>16500</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>MAX® 10 FPGA 10M50 (E144) 10M50SAE144C8G
+MAX® II CPLD EPM570 EPM570GF100I5N</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>Freeze architecture/BOM and evaluation plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>006Ui000020LXPl</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>HONEYWELL TECHNOLOGY SOLUTIONS</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Define</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>46726</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>47422</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Aerospace</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="n">
+        <v>90000</v>
+      </c>
+      <c r="M11" s="3" t="n">
+        <v>22500</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Agilex? 3 FPGA C-Series 065 (B18A) A3CZ065BB18AI7S
+Agilex? 3 FPGA C-Series 025 (B18A) A3CZ025BB18AI7S
+MAX® 10 FPGA 10M16 (F256) 10M16DAF256C8G</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>Freeze architecture/BOM and evaluation plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>006Ui00001mhnhF</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>HONEYWELL TECHNOLOGY SOLUTIONS</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Industrial automation controller - Process manager</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>46356</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>45943</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>46671</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>25000</v>
+      </c>
+      <c r="M12" s="3" t="n">
+        <v>18750</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Cyclone® 10 GX FPGA 10CX220 (F780) 10CX220YF780E5G</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>Secure DW evidence and production handoff</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>006Ui00002JOB82</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Philips India Limited - Innovation Center</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>User interface hub for MRI</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Define</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>46418</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>46126</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>46721</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Medical</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M13" s="3" t="n">
+        <v>2500</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>MAX® 10 FPGA 10M08 (F484) 10M08DAF484C8G</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>Freeze architecture/BOM and evaluation plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Identify / outside open exports</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>006Ui000029qRcE</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>HONEYWELL AEROSPACE INDIA PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Weather Monitoring Radar</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Identify</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>46715</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>46076</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>47171</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Aerospace</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="M14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Agilex? 9 FPGA Direct RF-Series 014 (R17B) AGRW014R17B2I2V</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>Qualify use case, sponsor, budget and 0→25% gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Identify / outside open exports</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>006Ui00002cUF9E</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>JUNIPER NETWORKS</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>CPU Interface Card_PQC</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Identify</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>46750</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>46222</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>47429</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Networking and Data Center OEM (IHV, ISV, SI, VAR)</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="n">
+        <v>600000</v>
+      </c>
+      <c r="M15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>Agilex? 3 FPGA C-Series 100 (M16A) A3CY100BM16AI6S</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>Qualify use case, sponsor, budget and 0→25% gate</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:P15"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Opportunities</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Peak Value</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Weighted Value</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026 open export</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>4125000</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>1031250</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>User-provided planning bucket; not derived from DWIN year</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2027 open export</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>4090045</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>1476511.25</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>User-provided planning bucket; includes some 2026 DWIN dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Qualified open combined</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>8215045</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>2507761.25</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>No overlapping opportunity IDs across uploaded exports</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Identify outside open exports</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Weather Radar and CPU Interface Card; 0% probability</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Total discovered portfolio</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>11815045</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>2507761.25</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Master-report universe</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="41" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Opportunity ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Opportunity</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Probability (%)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Design Win Date</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Peak Value</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Weighted Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>006Ui00001cftdL</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Outdu Mediatech Private Limited</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Intelligent Sense _Response Solution_AI</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Define</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>4125000</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>1031250</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -666,14 +2026,8 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="52" customWidth="1" min="14" max="14"/>
-    <col width="48" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -714,42 +2068,12 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Created Date</t>
+          <t>Peak Value</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Production Start Date</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Vertical</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Peak Value</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
           <t>Weighted Value</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Product Count</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Products</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Suggested Next Gate</t>
         </is>
       </c>
     </row>
@@ -759,59 +2083,35 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>006Ui00001cftdL</t>
+          <t>006Ui000029ckMz</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Outdu Mediatech Private Limited</t>
+          <t>JUNIPER NETWORKS</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Intelligent Sense _Response Solution_AI</t>
+          <t>CFPGA_PCIe Gen1</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Define</t>
+          <t>Develop</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>46316</v>
-      </c>
-      <c r="H2" s="4" t="n">
-        <v>45882</v>
-      </c>
-      <c r="I2" s="4" t="n">
-        <v>46679</v>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Broadcast</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="n">
-        <v>4125000</v>
-      </c>
-      <c r="L2" s="3" t="n">
-        <v>1031250</v>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>Agilex? 5 FPGA D-Series 064 (B32B) A5DD064AB32BI2V</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>Freeze architecture/BOM and evaluation plan</t>
-        </is>
+        <v>46437</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>900000</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>450000</v>
       </c>
     </row>
     <row r="3">
@@ -820,59 +2120,35 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>006Ui000029qRcE</t>
+          <t>006Ui00002SuI1A</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>HONEYWELL AEROSPACE INDIA PRIVATE LIMITED</t>
+          <t>Outdu Mediatech Private Limited</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Weather Monitoring Radar</t>
+          <t>Long Range Tracking System</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Identify</t>
+          <t>Define</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>46715</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>46076</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>47171</v>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Aerospace</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="L3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>Agilex? 9 FPGA Direct RF-Series 014 (R17B) AGRW014R17B2I2V</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>Qualify use case, sponsor, budget and 0→25% gate</t>
-        </is>
+        <v>46463</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>825000</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>206250</v>
       </c>
     </row>
     <row r="4">
@@ -881,59 +2157,35 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>006Ui000029ckMz</t>
+          <t>006Ui000023SJPy</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>JUNIPER NETWORKS</t>
+          <t>EMERSON INNOVATION CENTER - PUNE</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>CFPGA_PCIe Gen1</t>
+          <t>RX3i CEP002</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Develop</t>
+          <t>Define</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>46437</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>46075</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>46611</v>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Networking and Data Center OEM (IHV, ISV, SI, VAR)</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="n">
-        <v>900000</v>
-      </c>
-      <c r="L4" s="3" t="n">
-        <v>450000</v>
-      </c>
-      <c r="M4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>Cyclone® V GX FPGA 5CGXC7 (F31) 5CGXFC7D6F31I7N</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>Close validation plan and design-freeze evidence</t>
-        </is>
+        <v>46372</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>775000</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>193750</v>
       </c>
     </row>
     <row r="5">
@@ -942,17 +2194,17 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>006Ui00002SuI1A</t>
+          <t>006Ui00002VpuJp</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Outdu Mediatech Private Limited</t>
+          <t>GE HEALTHCARE</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Long Range Tracking System</t>
+          <t>Anesthesia Controller_X</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -964,37 +2216,13 @@
         <v>25</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>46463</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>46028</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>47017</v>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Broadcast</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="n">
-        <v>825000</v>
-      </c>
-      <c r="L5" s="3" t="n">
-        <v>206250</v>
-      </c>
-      <c r="M5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>Agilex? 5 FPGA D-Series 064 (B32B) A5DD064AB32BI3V</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>Freeze architecture/BOM and evaluation plan</t>
-        </is>
+        <v>46535</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>500000</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>125000</v>
       </c>
     </row>
     <row r="6">
@@ -1003,17 +2231,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>006Ui000023SJPy</t>
+          <t>006Ui00001rc0zI</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>EMERSON INNOVATION CENTER - PUNE</t>
+          <t>GE HEALTHCARE</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>RX3i CEP002</t>
+          <t>CT Scanner_DCB</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1025,38 +2253,13 @@
         <v>25</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>46372</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>46044</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>46491</v>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="n">
-        <v>775000</v>
-      </c>
-      <c r="L6" s="3" t="n">
-        <v>193750</v>
-      </c>
-      <c r="M6" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>Agilex? 3 FPGA C-Series 100 (B23C) A3CW100BB23CI6S
-Cyclone® V ST FPGA 5CSTD5 (F31) 5CSTFD5D5F31I7N</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>Freeze architecture/BOM and evaluation plan</t>
-        </is>
+        <v>46575</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>400045</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>100011.25</v>
       </c>
     </row>
     <row r="7">
@@ -1065,59 +2268,35 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>006Ui00002cUF9E</t>
+          <t>006Ui00001YL1Wo</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>JUNIPER NETWORKS</t>
+          <t>Philips India Limited - Innovation Center</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>CPU Interface Card_PQC</t>
+          <t>XSC/CT Scanner</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Identify</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>46750</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>46222</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>47429</v>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Networking and Data Center OEM (IHV, ISV, SI, VAR)</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="n">
-        <v>600000</v>
-      </c>
-      <c r="L7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>Agilex? 3 FPGA C-Series 100 (M16A) A3CY100BM16AI6S</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>Qualify use case, sponsor, budget and 0→25% gate</t>
-        </is>
+        <v>46276</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>270000</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>202500</v>
       </c>
     </row>
     <row r="8">
@@ -1126,59 +2305,35 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>006Ui00002VpuJp</t>
+          <t>006Ui00001nEdch</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>GE HEALTHCARE</t>
+          <t>HONEYWELL TECHNOLOGY SOLUTIONS</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Anesthesia Controller_X</t>
+          <t>micro vapour cooling system - VCS</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Define</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>46535</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>46189</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>46764</v>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Medical</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="n">
-        <v>500000</v>
-      </c>
-      <c r="L8" s="3" t="n">
-        <v>125000</v>
-      </c>
-      <c r="M8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>Agilex? 5 FPGA E-Series 028B (B23A) A5ED028BB23AI5S</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>Freeze architecture/BOM and evaluation plan</t>
-        </is>
+        <v>46539</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>185000</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>138750</v>
       </c>
     </row>
     <row r="9">
@@ -1187,7 +2342,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>006Ui00001rc0zI</t>
+          <t>006Ui00001YKvSK</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1197,7 +2352,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>CT Scanner_DCB</t>
+          <t>SP-PDU CONTROL BOARD</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1206,41 +2361,16 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>46575</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>45972</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>47296</v>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Medical</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="n">
-        <v>400045</v>
-      </c>
-      <c r="L9" s="3" t="n">
-        <v>100011.25</v>
-      </c>
-      <c r="M9" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>Agilex? 3 FPGA C-Series 065 (B18A) A3CY065BB18AE6S
-Cyclone® 10 GX FPGA 10CX150 (F672) 10CX150YF672E5G</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>Freeze architecture/BOM and evaluation plan</t>
-        </is>
+        <v>46351</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>110000</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>16500</v>
       </c>
     </row>
     <row r="10">
@@ -1249,59 +2379,35 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>006Ui00001YL1Wo</t>
+          <t>006Ui000020LXPl</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Philips India Limited - Innovation Center</t>
+          <t>HONEYWELL TECHNOLOGY SOLUTIONS</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>XSC/CT Scanner</t>
+          <t>CMU</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Define</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>45770</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>46345</v>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>Medical</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="n">
-        <v>270000</v>
-      </c>
-      <c r="L10" s="3" t="n">
-        <v>202500</v>
-      </c>
-      <c r="M10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>Cyclone® 10 LP FPGA 10CL120 (F780) 10CL120YF780C8G</t>
-        </is>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>Secure DW evidence and production handoff</t>
-        </is>
+        <v>46726</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>90000</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>22500</v>
       </c>
     </row>
     <row r="11">
@@ -1310,7 +2416,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>006Ui00001nEdch</t>
+          <t>006Ui00001mhnhF</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1320,7 +2426,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>micro vapour cooling system - VCS</t>
+          <t>Industrial automation controller - Process manager</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1332,38 +2438,13 @@
         <v>75</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>46539</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>45945</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>46741</v>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>Aerospace</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="n">
-        <v>185000</v>
-      </c>
-      <c r="L11" s="3" t="n">
-        <v>138750</v>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>MAX® 10 FPGA 10M04 (U324) 10M04SAU324I7G
-MAX® 10 FPGA 10M02 (U169) 10M02SCU169A7G</t>
-        </is>
-      </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>Secure DW evidence and production handoff</t>
-        </is>
+        <v>46356</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>25000</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>18750</v>
       </c>
     </row>
     <row r="12">
@@ -1372,17 +2453,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>006Ui00001YKvSK</t>
+          <t>006Ui00002JOB82</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>GE HEALTHCARE</t>
+          <t>Philips India Limited - Innovation Center</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>SP-PDU CONTROL BOARD</t>
+          <t>User interface hub for MRI</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1391,235 +2472,25 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>46351</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>45732</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>46806</v>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>Medical</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="n">
-        <v>110000</v>
-      </c>
-      <c r="L12" s="3" t="n">
-        <v>16500</v>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>MAX® 10 FPGA 10M50 (E144) 10M50SAE144C8G
-MAX® II CPLD EPM570 EPM570GF100I5N</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>Freeze architecture/BOM and evaluation plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>006Ui000020LXPl</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>HONEYWELL TECHNOLOGY SOLUTIONS</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>CMU</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Define</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G13" s="4" t="n">
-        <v>46726</v>
-      </c>
-      <c r="H13" s="4" t="n">
-        <v>46113</v>
-      </c>
-      <c r="I13" s="4" t="n">
-        <v>47422</v>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Aerospace</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="n">
-        <v>90000</v>
-      </c>
-      <c r="L13" s="3" t="n">
-        <v>22500</v>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>Agilex? 3 FPGA C-Series 065 (B18A) A3CZ065BB18AI7S
-Agilex? 3 FPGA C-Series 025 (B18A) A3CZ025BB18AI7S
-MAX® 10 FPGA 10M16 (F256) 10M16DAF256C8G</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>Freeze architecture/BOM and evaluation plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>006Ui00001mhnhF</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>HONEYWELL TECHNOLOGY SOLUTIONS</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Industrial automation controller - Process manager</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="G14" s="4" t="n">
-        <v>46356</v>
-      </c>
-      <c r="H14" s="4" t="n">
-        <v>45943</v>
-      </c>
-      <c r="I14" s="4" t="n">
-        <v>46671</v>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="n">
-        <v>25000</v>
-      </c>
-      <c r="L14" s="3" t="n">
-        <v>18750</v>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>Cyclone® 10 GX FPGA 10CX220 (F780) 10CX220YF780E5G</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>Secure DW evidence and production handoff</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>006Ui00002JOB82</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Philips India Limited - Innovation Center</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>User interface hub for MRI</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Define</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G15" s="4" t="n">
         <v>46418</v>
       </c>
-      <c r="H15" s="4" t="n">
-        <v>46126</v>
-      </c>
-      <c r="I15" s="4" t="n">
-        <v>46721</v>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>Medical</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="n">
+      <c r="H12" s="3" t="n">
         <v>10000</v>
       </c>
-      <c r="L15" s="3" t="n">
+      <c r="I12" s="3" t="n">
         <v>2500</v>
       </c>
-      <c r="M15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>MAX® 10 FPGA 10M08 (F484) 10M08DAF484C8G</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>Freeze architecture/BOM and evaluation plan</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O15"/>
+  <autoFilter ref="A1:I12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1838,7 +2709,7 @@
           <t>Agilex? 3 FPGA C-Series 100 (B23C) A3CW100BB23CI6S</t>
         </is>
       </c>
-      <c r="T2" s="2" t="n">
+      <c r="T2" s="3" t="n">
         <v>100000</v>
       </c>
     </row>
@@ -1928,7 +2799,7 @@
           <t>Cyclone® V ST FPGA 5CSTD5 (F31) 5CSTFD5D5F31I7N</t>
         </is>
       </c>
-      <c r="T3" s="2" t="n">
+      <c r="T3" s="3" t="n">
         <v>675000</v>
       </c>
     </row>
@@ -2018,7 +2889,7 @@
           <t>MAX® 10 FPGA 10M50 (E144) 10M50SAE144C8G</t>
         </is>
       </c>
-      <c r="T4" s="2" t="n">
+      <c r="T4" s="3" t="n">
         <v>80000</v>
       </c>
     </row>
@@ -2108,7 +2979,7 @@
           <t>MAX® II CPLD EPM570 EPM570GF100I5N</t>
         </is>
       </c>
-      <c r="T5" s="2" t="n">
+      <c r="T5" s="3" t="n">
         <v>30000</v>
       </c>
     </row>
@@ -2194,7 +3065,7 @@
           <t>Agilex? 3 FPGA C-Series 065 (B18A) A3CY065BB18AE6S</t>
         </is>
       </c>
-      <c r="T6" s="2" t="n">
+      <c r="T6" s="3" t="n">
         <v>45</v>
       </c>
     </row>
@@ -2280,7 +3151,7 @@
           <t>Cyclone® 10 GX FPGA 10CX150 (F672) 10CX150YF672E5G</t>
         </is>
       </c>
-      <c r="T7" s="2" t="n">
+      <c r="T7" s="3" t="n">
         <v>400000</v>
       </c>
     </row>
@@ -2368,7 +3239,7 @@
           <t>Agilex? 5 FPGA E-Series 028B (B23A) A5ED028BB23AI5S</t>
         </is>
       </c>
-      <c r="T8" s="2" t="n">
+      <c r="T8" s="3" t="n">
         <v>500000</v>
       </c>
     </row>
@@ -2456,7 +3327,7 @@
           <t>Cyclone® 10 GX FPGA 10CX220 (F780) 10CX220YF780E5G</t>
         </is>
       </c>
-      <c r="T9" s="2" t="n">
+      <c r="T9" s="3" t="n">
         <v>25000</v>
       </c>
     </row>
@@ -2544,7 +3415,7 @@
           <t>MAX® 10 FPGA 10M04 (U324) 10M04SAU324I7G</t>
         </is>
       </c>
-      <c r="T10" s="2" t="n">
+      <c r="T10" s="3" t="n">
         <v>160000</v>
       </c>
     </row>
@@ -2632,7 +3503,7 @@
           <t>MAX® 10 FPGA 10M02 (U169) 10M02SCU169A7G</t>
         </is>
       </c>
-      <c r="T11" s="2" t="n">
+      <c r="T11" s="3" t="n">
         <v>25000</v>
       </c>
     </row>
@@ -2718,7 +3589,7 @@
           <t>Agilex? 3 FPGA C-Series 065 (B18A) A3CZ065BB18AI7S</t>
         </is>
       </c>
-      <c r="T12" s="2" t="n">
+      <c r="T12" s="3" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2804,7 +3675,7 @@
           <t>Agilex? 3 FPGA C-Series 025 (B18A) A3CZ025BB18AI7S</t>
         </is>
       </c>
-      <c r="T13" s="2" t="n">
+      <c r="T13" s="3" t="n">
         <v>30000</v>
       </c>
     </row>
@@ -2890,7 +3761,7 @@
           <t>MAX® 10 FPGA 10M16 (F256) 10M16DAF256C8G</t>
         </is>
       </c>
-      <c r="T14" s="2" t="n">
+      <c r="T14" s="3" t="n">
         <v>10000</v>
       </c>
     </row>
@@ -2980,7 +3851,7 @@
           <t>Agilex? 9 FPGA Direct RF-Series 014 (R17B) AGRW014R17B2I2V</t>
         </is>
       </c>
-      <c r="T15" s="2" t="n">
+      <c r="T15" s="3" t="n">
         <v>3000000</v>
       </c>
     </row>
@@ -3068,7 +3939,7 @@
           <t>Cyclone® V GX FPGA 5CGXC7 (F31) 5CGXFC7D6F31I7N</t>
         </is>
       </c>
-      <c r="T16" s="2" t="n">
+      <c r="T16" s="3" t="n">
         <v>900000</v>
       </c>
     </row>
@@ -3156,7 +4027,7 @@
           <t>Agilex? 3 FPGA C-Series 100 (M16A) A3CY100BM16AI6S</t>
         </is>
       </c>
-      <c r="T17" s="2" t="n">
+      <c r="T17" s="3" t="n">
         <v>600000</v>
       </c>
     </row>
@@ -3246,7 +4117,7 @@
           <t>Agilex? 5 FPGA D-Series 064 (B32B) A5DD064AB32BI2V</t>
         </is>
       </c>
-      <c r="T18" s="2" t="n">
+      <c r="T18" s="3" t="n">
         <v>4125000</v>
       </c>
     </row>
@@ -3334,7 +4205,7 @@
           <t>Agilex? 5 FPGA D-Series 064 (B32B) A5DD064AB32BI3V</t>
         </is>
       </c>
-      <c r="T19" s="2" t="n">
+      <c r="T19" s="3" t="n">
         <v>825000</v>
       </c>
     </row>
@@ -3422,7 +4293,7 @@
           <t>Cyclone® 10 LP FPGA 10CL120 (F780) 10CL120YF780C8G</t>
         </is>
       </c>
-      <c r="T20" s="2" t="n">
+      <c r="T20" s="3" t="n">
         <v>270000</v>
       </c>
     </row>
@@ -3512,7 +4383,7 @@
           <t>MAX® 10 FPGA 10M08 (F484) 10M08DAF484C8G</t>
         </is>
       </c>
-      <c r="T21" s="2" t="n">
+      <c r="T21" s="3" t="n">
         <v>10000</v>
       </c>
     </row>
@@ -3522,7 +4393,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4071,7 +4942,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add account coverage and support execution evidence
Co-authored-by: Sahil Patni <sahilpat28@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/qbr/output/Sahil_QBR_Pipeline_Summary.xlsx
+++ b/qbr/output/Sahil_QBR_Pipeline_Summary.xlsx
@@ -12,19 +12,25 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline Reconciliation" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Pipeline 2026" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Pipeline 2027" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sahil Line Items" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market References" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joint GTM Plan" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account Coverage" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allocation Roster" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External Support Issues" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sahil Line Items" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market References" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joint GTM Plan" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Executive Summary'!$A$1:$C$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Executive Summary'!$A$1:$C$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Opportunities'!$A$1:$Q$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pipeline Reconciliation'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Open Pipeline 2026'!$A$1:$J$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Open Pipeline 2027'!$A$1:$J$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sahil Line Items'!$A$1:$T$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Market References'!$A$1:$E$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Joint GTM Plan'!$A$1:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Account Coverage'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Allocation Roster'!$A$1:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'External Support Issues'!$A$1:$G$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Sahil Line Items'!$A$1:$T$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Market References'!$A$1:$E$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Joint GTM Plan'!$A$1:$F$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,10 +462,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="44" customWidth="1" min="3" max="3"/>
   </cols>
@@ -711,39 +717,883 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026 annual target</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>INPUT REQUIRED</t>
-        </is>
+          <t>External support issue threads</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>16</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Not present in source</t>
+          <t>Distinct substantive external email threads, 15 May–28 Jul 2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>Explicitly resolved support threads</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Closure explicitly recorded in supplied summaries</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026 annual target</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>INPUT REQUIRED</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Not present in source</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>YTD actual achievement</t>
         </is>
       </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>INPUT REQUIRED</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Not present in source</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C20"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="37" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Accessed</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Use</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>International Federation of Robotics, World Robotics 2025 press release</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://ifr.org/ifr-press-releases/news/global-robot-demand-in-factories-doubles-over-10-years</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Robotics market</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Rockwell Automation, 2025 State of Smart Manufacturing — APAC findings</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rockwellautomation.com/en-sg/company/news/press-releases/apac-sosm-2025.html</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Industrial / APAC market</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Interact Analysis, Machine Vision return-to-growth forecast, June 2025</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://interactanalysis.com/return-to-growth-forecast-for-machine-vision-in-2025-despite-us-tariffs/</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Machine-vision market</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Robotics Solutions Stack</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/fpga-solutions/robotics-solutions-stack</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Altera robotics</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Agilex 5 FPGA and SoC FPGA overview</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/products/fpga/agilex/5</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Altera Agilex 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>AMD, Kria KR260 robotics platform and Kria Robotics Stack</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amd.com/en/products/system-on-modules/kria/k26/robotics.html</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>AMD robotics</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Video and Vision Processing Suite</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/products/ip/po-3150/video-and-vision-processing-suite</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Altera video / vision</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>R8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Altera, FPGA AI Suite</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/products/development-tools/fpga-ai-suite</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Altera AI software</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>AMD, Kria KV260 Vision AI Starter Kit</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amd.com/en/products/system-on-modules/kria/k26/kv260-vision-starter-kit.html</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>AMD vision</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>R10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>AMD, Versal AI Edge Series</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amd.com/en/products/adaptive-socs-and-fpgas/versal/ai-edge-series.html</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>AMD AI portfolio</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>R11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Industrial solutions</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/fpga-solutions/industrial</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Altera industrial</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Agilex 5 SoC HPS features including three 2.5G TSN Ethernet MACs</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>https://docs.altera.com/r/docs/762191/current/agilextm-5-fpgas-and-socs-device-overview/additional-features-for-agilextm-5-socs</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Altera TSN / HPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>R13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>AMD, Industrial Networking solutions</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amd.com/en/solutions/industrial/industrial-networking.html</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>AMD industrial networking</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Agilex 5 Functional Safety</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>https://docs.altera.com/api/khub/documents/xhgkkZ1PZaLEHFnNiUlbNA/content</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Altera functional safety</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>AMD, Functional Safety</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amd.com/en/products/adaptive-socs-and-fpgas/technologies/functional-safety.html</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>AMD functional safety</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Agilex 3 FPGA and SoC FPGA overview</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/products/fpga/agilex/3</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Altera cost-optimized portfolio</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>R17</t>
+        </is>
+      </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>INPUT REQUIRED</t>
+          <t>AMD, Spartan UltraScale+ FPGA overview</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Not present in source</t>
+          <t>https://www.amd.com/en/products/adaptive-socs-and-fpgas/fpga/spartan-ultrascale-plus.html</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>AMD cost-optimized portfolio</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>R18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>AMD, Vitis unified software platform</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amd.com/en/products/software/adaptive-socs-and-fpgas/vitis.html</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>AMD development tools</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>R19</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Video Solutions Stack</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/fpga-solutions/video-solutions-stack</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Altera video solution stack</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>R20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Altera, Sensor Interfaces including Holoscan Sensor Bridge</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.altera.com/fpga-solutions/sensory-interfaces</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Altera Holoscan / sensor interfaces</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C18"/>
+  <autoFilter ref="A1:E21"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Workstream</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Commitment</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Due</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Proposed KPI</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Altera / Sahil</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Lead program, architecture, benchmarks and DFAE coordination</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Named and charter accepted</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>NAMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Arrow</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Name robotics/AI/camera-capable joint specialist</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>≥1 named specialist</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Macnica</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Name robotics/AI/camera-capable joint specialist</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>≥1 named specialist</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Readiness</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Joint tiger team</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Verify solution access, kits, skills and benchmark playbooks</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>46248</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>≥1 robotics + ≥1 camera/AI demo path</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Targeting</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Arrow + Macnica</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Create non-duplicated joint account map</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>30 accounts: 15 per distributor</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Engagement</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Joint tiger team</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Run segment workshops and launch evaluations</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>46326</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>12 workshops; 8 evaluations</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Conversion</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Sales + FAE + distis</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Advance evidence-backed opportunities</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>46387</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>6 qualified; 3 Develop/Design; 2 DWINs</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>PROPOSED</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3461,6 +4311,1349 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Qualified Open Value</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Outside-Export Value</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Support Threads</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Coverage Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Ciena</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>2230000</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Primary; five qualified network platforms</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Juniper / HPE</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>900000</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>600000</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Primary; PCIe/flash support plus qualified and Identify pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Philips</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>280000</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Primary; CT and MRI pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>GE HealthCare</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>1010045</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Primary; CT, anesthesia and power-control pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Outdu</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>4950000</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Primary; AI response and tracking pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Other strategic / supported</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Other strategic; MAX 10 GPIO support</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Other strategic / supported</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>337500</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Other strategic; Data Recorder sits outside uploaded open exports</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Other strategic / supported</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Honeywell Aerospace</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Other strategic; I/O support and Identify-stage radar</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Other strategic / supported</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Schneider</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Other strategic; no supplied pipeline/support thread in period</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Other strategic / supported</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Emerson</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>775000</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Other strategic; RX3i pipeline</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Allocation Date</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>DFAE</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>New FAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ADA</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ADG</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>08 Feb 2025</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Amol</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Sahil</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>ADE</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>ADG</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>08 Feb 2025</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Amol</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Sahil</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>DEAL</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Dehradun</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>ADG</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>08 Feb 2025</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Mayank</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Sahil</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>C-DOT</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Across India</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>COMM</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>08 Jan 2026</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Mayank / Amol</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Sahil</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ADG</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>08 Feb 2025</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Sumanth / Prasad</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Sahil</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>LRDE</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>ADG</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>08 Feb 2025</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Sumanth / Prasad</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Sahil</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ECON</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>OTHERS</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>08 Feb 2025</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Akash</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Sahil</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ADG</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>08 Feb 2025</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Akash</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Sahil</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>IRDE</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Dehradun</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>ADG</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>08 Feb 2025</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>TBH / Prasad</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Sahil</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Ghaziabad</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>ADG</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>08 Feb 2025</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>TBH / Prasad</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Sahil</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Machilipatnam</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>ADG</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>08 Feb 2025</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Sumanth</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Sahil</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Outdu</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>OTHERS</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>08 Jan 2026</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Sahil</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F13"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="54" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="76" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Customer / Partner</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Latest Activity</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Technical Outcome / Next Action</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Quartus Pro 24.1 SignalTap compilation slowdown</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>C-DOT</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>46164</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Tools / AI</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Reproduce with an example design and SignalTap; provide a cleaner debug path.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Reproduction required</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>LVDS SerDes + optical transceiver integration for TSE</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Macnica / external</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>46171</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>100 Mbps optical fit requires hardware adaptation; TSE LVDS path is 1G-oriented.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Feasibility validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Non-PTP drops with PTP residence-time update in LL 40GbE MAC</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Ceragon</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>46161</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Trigger isolated to residence-time update control, narrowing MAC-level debug.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Debug narrowed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>MAX 10 DK-DEV-10M08E144-B GPIO feasibility</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>46198</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Device / I/O</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>44-signal fit is feasible subject to pin, bank-voltage, shared-circuit and level-shift checks.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Guidance provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Agilex 7 F-Tile TX MAC segmented-interface behavior</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>C-DOT</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>46191</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Clarified fixed latency, idle behavior and mid-frame valid-drop error handling.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Cyclone V PCIe MSI MsiReq_o not asserting</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>HPE</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>PCIe / Configuration</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Use MSI memory-write transaction flow rather than expecting MSIReq_o assertion.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Guidance provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>MAX 10 I/O utilization for 10M02SCE144A7G</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Honeywell Aerospace</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>46199</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Device / I/O</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>No fixed derating percentage; validate package and electrical constraints in Quartus.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Guidance provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>PTA 26.1 LPDDR5 frequency cap versus datasheet</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Vicharak</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Tools / AI</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Use 1866 MHz in Platform Designer and full Quartus power analysis pending PTA fix.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Workaround + escalation</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>FPGA AI Suite HL-JTAG memory and address-map issue</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Pantherun</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Tools / AI</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Use fabric DDR or expand the accessible bridge/span for F2SDRAM.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Guidance provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Agilex 7 custom-board bring-up and power sequencing</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>BEL / Macnica</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Board / Schematic</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Validate rail sequencing, pre-bias, waveforms, JTAG visibility and board captures first.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Bring-up investigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Agilex 3/5 schematic corrections before card release</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Qbit Labs / Arrow</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Board / Schematic</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Correct GTS bank power grouping before AI-Modem and TSN card release.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Release blocker found</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>ATUM Nano Ethernet failure after BSP regeneration</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Macnica / BEL Chennai</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>46206</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Reapply required manual driver edits after BSP regeneration, then rebuild.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Fix identified</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Agilex 7 core/HSSI rail topology for 3U VPX switch</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>BEL / Macnica</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>46210</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Board / Schematic</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Do not collapse regulators without current-sharing, transient and margin validation.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Validation required</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Dual-image Cyclone V GX flash update partitioning</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Juniper / HPE</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>46227</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>PCIe / Configuration</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Need a partition-safe primary-image update method; generated RPD spans full flash.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Method required</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Cyclone V PCIe MSI interrupt generation</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Juniper / HPE</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>PCIe / Configuration</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Implement MSI through the memory-write flow rather than MsiReq_o.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Guidance provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>SDR schematic-freeze pin and constraint blockers</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Macnica SDR program</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>46219</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Board / Schematic</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Close OPN mismatch, HPS UART, electrical constraints and pin handling before release.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Release blockers found</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G17"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:T28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5964,818 +8157,4 @@
   <autoFilter ref="A1:T28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="37" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Accessed</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Use</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>International Federation of Robotics, World Robotics 2025 press release</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://ifr.org/ifr-press-releases/news/global-robot-demand-in-factories-doubles-over-10-years</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Robotics market</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Rockwell Automation, 2025 State of Smart Manufacturing — APAC findings</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rockwellautomation.com/en-sg/company/news/press-releases/apac-sosm-2025.html</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Industrial / APAC market</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Interact Analysis, Machine Vision return-to-growth forecast, June 2025</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>https://interactanalysis.com/return-to-growth-forecast-for-machine-vision-in-2025-despite-us-tariffs/</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Machine-vision market</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>R4</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Altera, Robotics Solutions Stack</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.altera.com/fpga-solutions/robotics-solutions-stack</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Altera robotics</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>R5</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Altera, Agilex 5 FPGA and SoC FPGA overview</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.altera.com/products/fpga/agilex/5</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Altera Agilex 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>R6</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>AMD, Kria KR260 robotics platform and Kria Robotics Stack</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.amd.com/en/products/system-on-modules/kria/k26/robotics.html</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>AMD robotics</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>R7</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Altera, Video and Vision Processing Suite</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.altera.com/products/ip/po-3150/video-and-vision-processing-suite</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Altera video / vision</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>R8</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Altera, FPGA AI Suite</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.altera.com/products/development-tools/fpga-ai-suite</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Altera AI software</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>R9</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>AMD, Kria KV260 Vision AI Starter Kit</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.amd.com/en/products/system-on-modules/kria/k26/kv260-vision-starter-kit.html</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>AMD vision</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>R10</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>AMD, Versal AI Edge Series</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.amd.com/en/products/adaptive-socs-and-fpgas/versal/ai-edge-series.html</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>AMD AI portfolio</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>R11</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Altera, Industrial solutions</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.altera.com/fpga-solutions/industrial</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Altera industrial</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>R12</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Altera, Agilex 5 SoC HPS features including three 2.5G TSN Ethernet MACs</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>https://docs.altera.com/r/docs/762191/current/agilextm-5-fpgas-and-socs-device-overview/additional-features-for-agilextm-5-socs</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Altera TSN / HPS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>R13</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>AMD, Industrial Networking solutions</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.amd.com/en/solutions/industrial/industrial-networking.html</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>AMD industrial networking</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>R14</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Altera, Agilex 5 Functional Safety</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>https://docs.altera.com/api/khub/documents/xhgkkZ1PZaLEHFnNiUlbNA/content</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Altera functional safety</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>R15</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>AMD, Functional Safety</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>https://www.amd.com/en/products/adaptive-socs-and-fpgas/technologies/functional-safety.html</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>AMD functional safety</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>R16</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Altera, Agilex 3 FPGA and SoC FPGA overview</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>https://www.altera.com/products/fpga/agilex/3</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Altera cost-optimized portfolio</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>R17</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>AMD, Spartan UltraScale+ FPGA overview</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.amd.com/en/products/adaptive-socs-and-fpgas/fpga/spartan-ultrascale-plus.html</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>AMD cost-optimized portfolio</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>R18</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>AMD, Vitis unified software platform</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>https://www.amd.com/en/products/software/adaptive-socs-and-fpgas/vitis.html</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>AMD development tools</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>R19</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Altera, Video Solutions Stack</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.altera.com/fpga-solutions/video-solutions-stack</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Altera video solution stack</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>R20</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Altera, Sensor Interfaces including Holoscan Sensor Bridge</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>https://www.altera.com/fpga-solutions/sensory-interfaces</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Altera Holoscan / sensor interfaces</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E21"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Workstream</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Commitment</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Due</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Proposed KPI</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Team</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Altera / Sahil</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Lead program, architecture, benchmarks and DFAE coordination</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>46239</v>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Named and charter accepted</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>NAMED</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Team</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Arrow</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Name robotics/AI/camera-capable joint specialist</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>46239</v>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>≥1 named specialist</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Team</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Macnica</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Name robotics/AI/camera-capable joint specialist</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>46239</v>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>≥1 named specialist</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Readiness</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Joint tiger team</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Verify solution access, kits, skills and benchmark playbooks</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>46248</v>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>≥1 robotics + ≥1 camera/AI demo path</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Targeting</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Arrow + Macnica</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Create non-duplicated joint account map</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>46265</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>30 accounts: 15 per distributor</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Engagement</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Joint tiger team</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Run segment workshops and launch evaluations</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>46326</v>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>12 workshops; 8 evaluations</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Conversion</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Sales + FAE + distis</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Advance evidence-backed opportunities</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>46387</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>6 qualified; 3 Develop/Design; 2 DWINs</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSED</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F8"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Align QBR to Altera fiscal calendar
Co-authored-by: Sahil Patni <sahilpat28@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/qbr/output/Sahil_QBR_Pipeline_Summary.xlsx
+++ b/qbr/output/Sahil_QBR_Pipeline_Summary.xlsx
@@ -10,8 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline Reconciliation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Pipeline 2026" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Pipeline 2027" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Pipeline FY2026" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Pipeline FY2027" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account Coverage" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allocation Roster" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External Support Issues" sheetId="8" state="visible" r:id="rId8"/>
@@ -20,14 +20,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joint GTM Plan" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Executive Summary'!$A$1:$C$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Executive Summary'!$A$1:$C$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Opportunities'!$A$1:$Q$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pipeline Reconciliation'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Open Pipeline 2026'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Open Pipeline 2027'!$A$1:$J$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Open Pipeline FY2026'!$A$1:$J$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Open Pipeline FY2027'!$A$1:$J$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Account Coverage'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Allocation Roster'!$A$1:$F$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'External Support Issues'!$A$1:$G$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'External Support Issues'!$A$1:$H$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Sahil Line Items'!$A$1:$T$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Market References'!$A$1:$E$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Joint GTM Plan'!$A$1:$F$8</definedName>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -498,7 +498,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Combined uploaded 2026 + 2027 open exports</t>
+          <t>Combined uploaded FY2026 + FY2027 planning exports</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026 open-export opportunities</t>
+          <t>FY2026 open-export opportunities</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
@@ -543,14 +543,14 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>User-provided planning bucket</t>
+          <t>User-provided fiscal planning bucket</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026 open-export peak value</t>
+          <t>FY2026 open-export peak value</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
@@ -558,14 +558,14 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>User-provided planning bucket</t>
+          <t>User-provided fiscal planning bucket</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2027 open-export opportunities</t>
+          <t>FY2027 open-export opportunities</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
@@ -573,14 +573,14 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>User-provided planning bucket</t>
+          <t>User-provided fiscal planning bucket</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2027 open-export peak value</t>
+          <t>FY2027 open-export peak value</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
@@ -588,198 +588,305 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>User-provided planning bucket</t>
+          <t>User-provided fiscal planning bucket</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Identify outside open exports</t>
+          <t>Q4 FY2026 DWIN-dated opportunities</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Master-report opportunities absent from both open exports</t>
+          <t>Design Win Date from 01 Aug–31 Oct 2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Identify peak value</t>
+          <t>Q4 FY2026 DWIN-dated peak value</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>3600000</v>
+        <v>4951500</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>0% probability in master report</t>
+          <t>Scheduled date; not proof of achieved DWIN</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Other outside open exports</t>
+          <t>FY2027 DWIN-dated opportunities</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Non-Identify master opportunities absent from both exports</t>
+          <t>Design Win Date from 01 Nov 2026–31 Oct 2027</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Other outside peak value</t>
+          <t>FY2027 DWIN-dated peak value</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>337500</v>
+        <v>5403545</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Review reason for exclusion</t>
+          <t>Scheduled date; not proof of achieved DWIN</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Total discovered opportunities</t>
+          <t>Identify outside open exports</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Qualified open + outside-export plays</t>
+          <t>Master-report opportunities absent from both open exports</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Total discovered peak value</t>
+          <t>Identify peak value</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>14382545</v>
+        <v>3600000</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Qualified open + outside-export plays</t>
+          <t>0% probability in master report</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Reporting scope</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Sahil + Kasturi</t>
-        </is>
+          <t>Other outside open exports</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Only these two source Technical Owner values are included</t>
+          <t>Non-Identify master opportunities absent from both exports</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Product line items</t>
+          <t>Other outside peak value</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>27</v>
+        <v>337500</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Technical Owner = Sahil Patni or Kasturi Rangan</t>
+          <t>Review reason for exclusion</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>External support issue threads</t>
+          <t>Total discovered opportunities</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Distinct substantive external email threads, 15 May–28 Jul 2026</t>
+          <t>Qualified open + outside-export plays</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Explicitly resolved support threads</t>
+          <t>Total discovered peak value</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>1</v>
+        <v>14382545</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Closure explicitly recorded in supplied summaries</t>
+          <t>Qualified open + outside-export plays</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026 annual target</t>
+          <t>Reporting scope</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>INPUT REQUIRED</t>
+          <t>Sahil + Kasturi</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Not present in source</t>
+          <t>Only these two source Technical Owner values are included</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>FAE team start</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>46174</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Sahil joined the FAE team on 01 Jun 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Fiscal calendar</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>01 Nov–31 Oct</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>FY2026 Q4 = Aug–Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Product line items</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Technical Owner = Sahil Patni or Kasturi Rangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>External support issue threads</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Distinct substantive external email threads, 15 May–28 Jul 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Threads latest before FAE start</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Transition/pre-start context; FAE start = 01 Jun 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Explicitly resolved support threads</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Closure explicitly recorded in supplied summaries</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>FY2026 annual target</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>INPUT REQUIRED</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Not present in source</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>YTD actual achievement</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>INPUT REQUIRED</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Not present in source</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C20"/>
+  <autoFilter ref="A1:C27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1342,7 +1449,7 @@
   <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="62" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -1565,7 +1672,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Conversion</t>
+          <t>Q4 FY2026 conversion</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1579,7 +1686,7 @@
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>46387</v>
+        <v>46326</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -1719,7 +1826,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>FY2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1790,7 +1897,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1861,7 +1968,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1932,7 +2039,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2004,7 +2111,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2075,7 +2182,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2146,7 +2253,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2217,7 +2324,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2288,7 +2395,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2359,7 +2466,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2431,7 +2538,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2502,7 +2609,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2574,7 +2681,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>FY2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2645,7 +2752,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2716,7 +2823,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -2788,7 +2895,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2861,7 +2968,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -2932,7 +3039,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>FY2027</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -3145,7 +3252,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Outside uploaded 2026/2027</t>
+          <t>Outside uploaded FY2026/FY2027</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3262,7 +3369,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026 open export</t>
+          <t>FY2026 open export</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -3276,14 +3383,14 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>User-provided planning bucket; not derived from DWIN year</t>
+          <t>User-provided fiscal planning bucket; membership retained from export</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2027 open export</t>
+          <t>FY2027 open export</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -3297,7 +3404,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>User-provided planning bucket; includes some 2026 DWIN dates</t>
+          <t>User-provided fiscal planning bucket; membership retained from export</t>
         </is>
       </c>
     </row>
@@ -5065,7 +5172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5073,8 +5180,9 @@
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="76" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="76" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5100,15 +5208,20 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>FAE Context</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Theme</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Technical Outcome / Next Action</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -5133,15 +5246,20 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>Pre-start / transition</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>Tools / AI</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Reproduce with an example design and SignalTap; provide a cleaner debug path.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Reproduction required</t>
         </is>
@@ -5166,15 +5284,20 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>Pre-start / transition</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>Networking</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>100 Mbps optical fit requires hardware adaptation; TSE LVDS path is 1G-oriented.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Feasibility validation</t>
         </is>
@@ -5199,15 +5322,20 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>Pre-start / transition</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>Networking</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Trigger isolated to residence-time update control, narrowing MAC-level debug.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Debug narrowed</t>
         </is>
@@ -5232,15 +5360,20 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>Device / I/O</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>44-signal fit is feasible subject to pin, bank-voltage, shared-circuit and level-shift checks.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Guidance provided</t>
         </is>
@@ -5265,15 +5398,20 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>Networking</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Clarified fixed latency, idle behavior and mid-frame valid-drop error handling.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -5298,15 +5436,20 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>PCIe / Configuration</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Use MSI memory-write transaction flow rather than expecting MSIReq_o assertion.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Guidance provided</t>
         </is>
@@ -5331,15 +5474,20 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>Device / I/O</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>No fixed derating percentage; validate package and electrical constraints in Quartus.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Guidance provided</t>
         </is>
@@ -5364,15 +5512,20 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
           <t>Tools / AI</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Use 1866 MHz in Platform Designer and full Quartus power analysis pending PTA fix.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Workaround + escalation</t>
         </is>
@@ -5397,15 +5550,20 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>Tools / AI</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Use fabric DDR or expand the accessible bridge/span for F2SDRAM.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Guidance provided</t>
         </is>
@@ -5430,15 +5588,20 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
           <t>Board / Schematic</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Validate rail sequencing, pre-bias, waveforms, JTAG visibility and board captures first.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Bring-up investigation</t>
         </is>
@@ -5463,15 +5626,20 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
           <t>Board / Schematic</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Correct GTS bank power grouping before AI-Modem and TSN card release.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Release blocker found</t>
         </is>
@@ -5496,15 +5664,20 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>Networking</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Reapply required manual driver edits after BSP regeneration, then rebuild.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Fix identified</t>
         </is>
@@ -5529,15 +5702,20 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>Board / Schematic</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Do not collapse regulators without current-sharing, transient and margin validation.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Validation required</t>
         </is>
@@ -5562,15 +5740,20 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
           <t>PCIe / Configuration</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Need a partition-safe primary-image update method; generated RPD spans full flash.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Method required</t>
         </is>
@@ -5595,15 +5778,20 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>PCIe / Configuration</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Implement MSI through the memory-write flow rather than MsiReq_o.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Guidance provided</t>
         </is>
@@ -5628,22 +5816,27 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
           <t>Board / Schematic</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Close OPN mismatch, HPS UART, electrical constraints and pin handling before release.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Release blockers found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G17"/>
+  <autoFilter ref="A1:H17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add FY2026 and FY2027 stage funnels
Co-authored-by: Sahil Patni <sahilpat28@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/qbr/output/Sahil_QBR_Pipeline_Summary.xlsx
+++ b/qbr/output/Sahil_QBR_Pipeline_Summary.xlsx
@@ -9,30 +9,32 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Pipeline Snapshot" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline Reconciliation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Pipeline FY2026" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Pipeline FY2027" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account Coverage" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allocation Roster" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External Support Issues" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sahil Line Items" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market References" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joint GTM Plan" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunity Stage Funnel" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline Reconciliation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Pipeline FY2026" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Pipeline FY2027" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account Coverage" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allocation Roster" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External Support Issues" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sahil Line Items" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market References" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Joint GTM Plan" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Executive Summary'!$A$1:$C$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Total Pipeline Snapshot'!$A$1:$I$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Opportunities'!$A$1:$Q$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pipeline Reconciliation'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Open Pipeline FY2026'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Open Pipeline FY2027'!$A$1:$J$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Account Coverage'!$A$1:$F$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Allocation Roster'!$A$1:$F$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'External Support Issues'!$A$1:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Sahil Line Items'!$A$1:$T$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Market References'!$A$1:$E$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Joint GTM Plan'!$A$1:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Opportunity Stage Funnel'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Opportunities'!$A$1:$Q$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Pipeline Reconciliation'!$A$1:$E$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Open Pipeline FY2026'!$A$1:$J$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Open Pipeline FY2027'!$A$1:$J$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Account Coverage'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Allocation Roster'!$A$1:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'External Support Issues'!$A$1:$H$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Sahil Line Items'!$A$1:$T$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Market References'!$A$1:$E$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Joint GTM Plan'!$A$1:$F$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -40,9 +42,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -82,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -94,6 +97,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -989,6 +995,681 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="54" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="76" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Customer / Partner</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Latest Activity</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>FAE Context</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Technical Outcome / Next Action</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Quartus Pro 24.1 SignalTap compilation slowdown</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>C-DOT</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>46164</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Pre-start / transition</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Tools / AI</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Reproduce with an example design and SignalTap; provide a cleaner debug path.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Reproduction required</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>LVDS SerDes + optical transceiver integration for TSE</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Macnica / external</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>46171</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Pre-start / transition</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>100 Mbps optical fit requires hardware adaptation; TSE LVDS path is 1G-oriented.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Feasibility validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Non-PTP drops with PTP residence-time update in LL 40GbE MAC</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Ceragon</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>46161</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Pre-start / transition</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Trigger isolated to residence-time update control, narrowing MAC-level debug.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Debug narrowed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>MAX 10 DK-DEV-10M08E144-B GPIO feasibility</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>46198</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Device / I/O</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>44-signal fit is feasible subject to pin, bank-voltage, shared-circuit and level-shift checks.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Guidance provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Agilex 7 F-Tile TX MAC segmented-interface behavior</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>C-DOT</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>46191</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Clarified fixed latency, idle behavior and mid-frame valid-drop error handling.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Cyclone V PCIe MSI MsiReq_o not asserting</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>HPE</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>PCIe / Configuration</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Use MSI memory-write transaction flow rather than expecting MSIReq_o assertion.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Guidance provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>MAX 10 I/O utilization for 10M02SCE144A7G</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Honeywell Aerospace</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>46199</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Device / I/O</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>No fixed derating percentage; validate package and electrical constraints in Quartus.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Guidance provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>PTA 26.1 LPDDR5 frequency cap versus datasheet</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Vicharak</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Tools / AI</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Use 1866 MHz in Platform Designer and full Quartus power analysis pending PTA fix.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Workaround + escalation</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>FPGA AI Suite HL-JTAG memory and address-map issue</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Pantherun</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Tools / AI</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Use fabric DDR or expand the accessible bridge/span for F2SDRAM.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Guidance provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Agilex 7 custom-board bring-up and power sequencing</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>BEL / Macnica</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Board / Schematic</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Validate rail sequencing, pre-bias, waveforms, JTAG visibility and board captures first.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Bring-up investigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Agilex 3/5 schematic corrections before card release</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Qbit Labs / Arrow</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Board / Schematic</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Correct GTS bank power grouping before AI-Modem and TSN card release.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Release blocker found</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>ATUM Nano Ethernet failure after BSP regeneration</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Macnica / BEL Chennai</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>46206</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Reapply required manual driver edits after BSP regeneration, then rebuild.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Fix identified</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Agilex 7 core/HSSI rail topology for 3U VPX switch</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>BEL / Macnica</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>46210</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Board / Schematic</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Do not collapse regulators without current-sharing, transient and margin validation.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Validation required</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Dual-image Cyclone V GX flash update partitioning</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Juniper / HPE</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>46227</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>PCIe / Configuration</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Need a partition-safe primary-image update method; generated RPD spans full flash.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Method required</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Cyclone V PCIe MSI interrupt generation</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Juniper / HPE</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>PCIe / Configuration</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Implement MSI through the memory-write flow rather than MsiReq_o.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Guidance provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>SDR schematic-freeze pin and constraint blockers</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Macnica SDR program</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>46219</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>FAE tenure</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Board / Schematic</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Close OPN mismatch, HPS UART, electrical constraints and pin handling before release.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Release blockers found</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H17"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:T28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1173,10 +1854,10 @@
           <t>Emerging</t>
         </is>
       </c>
-      <c r="M2" s="5" t="n">
+      <c r="M2" s="6" t="n">
         <v>46240</v>
       </c>
-      <c r="N2" s="5" t="n">
+      <c r="N2" s="6" t="n">
         <v>47609</v>
       </c>
       <c r="O2" s="2" t="n">
@@ -1259,7 +1940,7 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="M3" s="5" t="n">
+      <c r="M3" s="6" t="n">
         <v>45843</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -1347,7 +2028,7 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="M4" s="5" t="n">
+      <c r="M4" s="6" t="n">
         <v>45941</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -1405,7 +2086,7 @@
           <t>Define</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="6" t="n">
         <v>46245</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1433,7 +2114,7 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="M5" s="5" t="n">
+      <c r="M5" s="6" t="n">
         <v>45941</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -1521,7 +2202,7 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="M6" s="5" t="n">
+      <c r="M6" s="6" t="n">
         <v>45972</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -1609,10 +2290,10 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="M7" s="5" t="n">
+      <c r="M7" s="6" t="n">
         <v>45972</v>
       </c>
-      <c r="N7" s="5" t="n">
+      <c r="N7" s="6" t="n">
         <v>46457</v>
       </c>
       <c r="O7" s="2" t="n">
@@ -1665,7 +2346,7 @@
           <t>Define</t>
         </is>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G8" s="6" t="n">
         <v>46242</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1693,7 +2374,7 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="M8" s="5" t="n">
+      <c r="M8" s="6" t="n">
         <v>45972</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -2111,7 +2792,7 @@
           <t>Define</t>
         </is>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="6" t="n">
         <v>46575</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -2139,7 +2820,7 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="M13" s="5" t="n">
+      <c r="M13" s="6" t="n">
         <v>45972</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -2197,7 +2878,7 @@
           <t>Define</t>
         </is>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="G14" s="6" t="n">
         <v>46575</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -2225,7 +2906,7 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="M14" s="5" t="n">
+      <c r="M14" s="6" t="n">
         <v>45972</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -2318,7 +2999,7 @@
           <t>6/16/2026</t>
         </is>
       </c>
-      <c r="N15" s="5" t="n">
+      <c r="N15" s="6" t="n">
         <v>46764</v>
       </c>
       <c r="O15" s="2" t="n">
@@ -2406,7 +3087,7 @@
           <t>10/13/2025</t>
         </is>
       </c>
-      <c r="N16" s="5" t="n">
+      <c r="N16" s="6" t="n">
         <v>46671</v>
       </c>
       <c r="O16" s="2" t="n">
@@ -2459,7 +3140,7 @@
           <t>Design</t>
         </is>
       </c>
-      <c r="G17" s="5" t="n">
+      <c r="G17" s="6" t="n">
         <v>46539</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -2547,7 +3228,7 @@
           <t>Design</t>
         </is>
       </c>
-      <c r="G18" s="5" t="n">
+      <c r="G18" s="6" t="n">
         <v>46539</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -2635,7 +3316,7 @@
           <t>Define</t>
         </is>
       </c>
-      <c r="G19" s="5" t="n">
+      <c r="G19" s="6" t="n">
         <v>46726</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -2663,7 +3344,7 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="M19" s="5" t="n">
+      <c r="M19" s="6" t="n">
         <v>46113</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -2721,7 +3402,7 @@
           <t>Define</t>
         </is>
       </c>
-      <c r="G20" s="5" t="n">
+      <c r="G20" s="6" t="n">
         <v>46726</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -2749,7 +3430,7 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="M20" s="5" t="n">
+      <c r="M20" s="6" t="n">
         <v>46113</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -2807,7 +3488,7 @@
           <t>Define</t>
         </is>
       </c>
-      <c r="G21" s="5" t="n">
+      <c r="G21" s="6" t="n">
         <v>46726</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -2835,7 +3516,7 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="M21" s="5" t="n">
+      <c r="M21" s="6" t="n">
         <v>46113</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
@@ -3018,7 +3699,7 @@
           <t>2/22/2026</t>
         </is>
       </c>
-      <c r="N23" s="5" t="n">
+      <c r="N23" s="6" t="n">
         <v>46611</v>
       </c>
       <c r="O23" s="2" t="n">
@@ -3106,7 +3787,7 @@
           <t>7/19/2026</t>
         </is>
       </c>
-      <c r="N24" s="5" t="n">
+      <c r="N24" s="6" t="n">
         <v>47429</v>
       </c>
       <c r="O24" s="2" t="n">
@@ -3279,7 +3960,7 @@
           <t>Focused</t>
         </is>
       </c>
-      <c r="M26" s="5" t="n">
+      <c r="M26" s="6" t="n">
         <v>46028</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
@@ -3337,7 +4018,7 @@
           <t>Design</t>
         </is>
       </c>
-      <c r="G27" s="5" t="n">
+      <c r="G27" s="6" t="n">
         <v>46276</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -3494,7 +4175,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4043,7 +4724,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4444,6 +5125,301 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="31" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Fiscal Bucket</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Total Value</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Distinct Opportunities</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Source Rows</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Direct Value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Channel Value</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Distinct Direct Opportunities</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Distinct Channel Opportunities</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Value Share</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>FY2026</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Define</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>12655200</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>4252500</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>8402700</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>0.7297133664308326</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>FY2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Develop</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>3687500</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>3687500</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>0.2126254850744117</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>FY2026</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>0.05766114849475572</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>FY2027</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Define</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>55929710</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>4812545</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>51117165</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>0.8669967668433171</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>FY2027</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Develop</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>8100000</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>900000</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>7200000</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>0.1255624928402251</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>FY2027</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>480000</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>480000</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>0.007440740316457786</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6061,7 +7037,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6236,7 +7212,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6399,7 +7375,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7150,7 +8126,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7465,7 +8441,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7902,679 +8878,4 @@
   <autoFilter ref="A1:F13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="54" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="76" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Issue</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Customer / Partner</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Latest Activity</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>FAE Context</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Technical Outcome / Next Action</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Quartus Pro 24.1 SignalTap compilation slowdown</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>C-DOT</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>46164</v>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Pre-start / transition</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Tools / AI</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Reproduce with an example design and SignalTap; provide a cleaner debug path.</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Reproduction required</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>LVDS SerDes + optical transceiver integration for TSE</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Macnica / external</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>46171</v>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Pre-start / transition</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Networking</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>100 Mbps optical fit requires hardware adaptation; TSE LVDS path is 1G-oriented.</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Feasibility validation</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Non-PTP drops with PTP residence-time update in LL 40GbE MAC</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Ceragon</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>46161</v>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Pre-start / transition</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Networking</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Trigger isolated to residence-time update control, narrowing MAC-level debug.</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Debug narrowed</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>MAX 10 DK-DEV-10M08E144-B GPIO feasibility</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Siemens</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>46198</v>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>FAE tenure</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Device / I/O</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>44-signal fit is feasible subject to pin, bank-voltage, shared-circuit and level-shift checks.</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Guidance provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Agilex 7 F-Tile TX MAC segmented-interface behavior</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>C-DOT</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>46191</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>FAE tenure</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Networking</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Clarified fixed latency, idle behavior and mid-frame valid-drop error handling.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Resolved</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Cyclone V PCIe MSI MsiReq_o not asserting</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>HPE</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>46202</v>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>FAE tenure</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>PCIe / Configuration</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Use MSI memory-write transaction flow rather than expecting MSIReq_o assertion.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Guidance provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>MAX 10 I/O utilization for 10M02SCE144A7G</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Honeywell Aerospace</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>46199</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>FAE tenure</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Device / I/O</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>No fixed derating percentage; validate package and electrical constraints in Quartus.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Guidance provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>PTA 26.1 LPDDR5 frequency cap versus datasheet</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Vicharak</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>46231</v>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>FAE tenure</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Tools / AI</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Use 1866 MHz in Platform Designer and full Quartus power analysis pending PTA fix.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Workaround + escalation</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>FPGA AI Suite HL-JTAG memory and address-map issue</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Pantherun</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>46218</v>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>FAE tenure</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Tools / AI</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Use fabric DDR or expand the accessible bridge/span for F2SDRAM.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Guidance provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Agilex 7 custom-board bring-up and power sequencing</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>BEL / Macnica</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>46230</v>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>FAE tenure</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Board / Schematic</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Validate rail sequencing, pre-bias, waveforms, JTAG visibility and board captures first.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Bring-up investigation</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Agilex 3/5 schematic corrections before card release</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Qbit Labs / Arrow</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>46218</v>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>FAE tenure</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Board / Schematic</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Correct GTS bank power grouping before AI-Modem and TSN card release.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Release blocker found</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>ATUM Nano Ethernet failure after BSP regeneration</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Macnica / BEL Chennai</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="n">
-        <v>46206</v>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>FAE tenure</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Networking</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Reapply required manual driver edits after BSP regeneration, then rebuild.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Fix identified</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Agilex 7 core/HSSI rail topology for 3U VPX switch</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>BEL / Macnica</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>46210</v>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>FAE tenure</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Board / Schematic</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Do not collapse regulators without current-sharing, transient and margin validation.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Validation required</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Dual-image Cyclone V GX flash update partitioning</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Juniper / HPE</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="n">
-        <v>46227</v>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>FAE tenure</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>PCIe / Configuration</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Need a partition-safe primary-image update method; generated RPD spans full flash.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Method required</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Cyclone V PCIe MSI interrupt generation</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Juniper / HPE</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>46217</v>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>FAE tenure</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>PCIe / Configuration</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Implement MSI through the memory-write flow rather than MsiReq_o.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Guidance provided</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>SDR schematic-freeze pin and constraint blockers</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Macnica SDR program</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>46219</v>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>FAE tenure</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Board / Schematic</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Close OPN mismatch, HPS UART, electrical constraints and pin handling before release.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Release blockers found</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:H17"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>